<commit_message>
🚀 Actualización final: Logo Base64, Regla de Asistencia 80% y Fix de reportes administrativos
</commit_message>
<xml_diff>
--- a/data/journey.xlsx
+++ b/data/journey.xlsx
@@ -3,7 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Base de Datos" sheetId="1" r:id="rId1"/>
+    <sheet name="Estudiantes" sheetId="1" r:id="rId1"/>
+    <sheet name="Docentes" sheetId="2" r:id="rId2"/>
+    <sheet name="Administrativos" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -397,531 +399,935 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:F31"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Programa</v>
+        <v>Usuario</v>
       </c>
       <c r="B1" t="str">
+        <v>Contraseña</v>
+      </c>
+      <c r="C1" t="str">
         <v>Estudiante</v>
       </c>
-      <c r="C1" t="str">
-        <v>Usuario estudiante</v>
-      </c>
       <c r="D1" t="str">
-        <v>Contraseña estudiante</v>
+        <v>Programa asignado</v>
       </c>
       <c r="E1" t="str">
-        <v>Docente</v>
+        <v>Código programa</v>
       </c>
       <c r="F1" t="str">
-        <v>Usuario Docente</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Contraseña doc</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Materia</v>
+        <v>Correo</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Gestión De Turismo De Reuniones, Incentivos Y Convenciones</v>
+        <v>39789871</v>
       </c>
       <c r="B2" t="str">
-        <v>Ximena</v>
+        <v>Est1Al</v>
       </c>
       <c r="C2" t="str">
-        <v>Est12</v>
+        <v>Alda Salomé Grajales Lemos</v>
       </c>
       <c r="D2" t="str">
-        <v>789</v>
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E2" t="str">
-        <v>Edgar Blanco</v>
+        <v>DIo1</v>
       </c>
       <c r="F2" t="str">
-        <v>Doc01</v>
-      </c>
-      <c r="G2" t="str">
-        <v>123</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Presupuestos</v>
+        <v>salome.grajales@gmail.com</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Gestión Estratégica de la experiencia</v>
+        <v>1024527737</v>
       </c>
       <c r="B3" t="str">
-        <v>Katerine</v>
+        <v>Est2Al</v>
       </c>
       <c r="C3" t="str">
-        <v>Est06</v>
+        <v>Alberto Vargas Azuaje</v>
       </c>
       <c r="D3" t="str">
-        <v>789</v>
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E3" t="str">
-        <v>Edgar Blanco</v>
+        <v>DIo1</v>
       </c>
       <c r="F3" t="str">
-        <v>Doc01</v>
-      </c>
-      <c r="G3" t="str">
-        <v>123</v>
-      </c>
-      <c r="H3" t="str">
-        <v>Presupuestos</v>
+        <v>alberto.vargas@thesomos.com</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Marketing Digital para hoteles</v>
+        <v>16932775</v>
       </c>
       <c r="B4" t="str">
-        <v>Eliana</v>
+        <v>Est3An</v>
       </c>
       <c r="C4" t="str">
-        <v>Est11</v>
+        <v>Andrés Felipe Vallejo Mosquera</v>
       </c>
       <c r="D4" t="str">
-        <v>789</v>
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E4" t="str">
-        <v>Edgar Blanco</v>
+        <v>DIo1</v>
       </c>
       <c r="F4" t="str">
-        <v>Doc01</v>
-      </c>
-      <c r="G4" t="str">
-        <v>123</v>
-      </c>
-      <c r="H4" t="str">
-        <v>Presupuestos</v>
+        <v>avallejo@metro-op.com</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Sales Upgrade: Dominando Las Tecnologías</v>
+        <v>1151950133</v>
       </c>
       <c r="B5" t="str">
-        <v>David</v>
+        <v>Est4Ay</v>
       </c>
       <c r="C5" t="str">
-        <v>Est01</v>
+        <v>Aylén Alejandra Pérez Cortes</v>
       </c>
       <c r="D5" t="str">
-        <v>987</v>
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E5" t="str">
-        <v>Edgar Blanco</v>
+        <v>DIo1</v>
       </c>
       <c r="F5" t="str">
-        <v>Doc01</v>
-      </c>
-      <c r="G5" t="str">
-        <v>123</v>
-      </c>
-      <c r="H5" t="str">
-        <v>Presupuestos</v>
+        <v>financiero.hamptoncali@metro-op.com</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>De La Gestión De Eventos Sostenibles A La Gestión Sostenible De Eventos</v>
+        <v>1000383477</v>
       </c>
       <c r="B6" t="str">
-        <v>Claudia</v>
+        <v>Est5Ca</v>
       </c>
       <c r="C6" t="str">
-        <v>Est03</v>
+        <v>Camila Andrea Cárdenas Lara</v>
       </c>
       <c r="D6" t="str">
-        <v>789</v>
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E6" t="str">
-        <v>Eduardo Pacheco</v>
+        <v>DIo1</v>
       </c>
       <c r="F6" t="str">
-        <v>Doc02</v>
-      </c>
-      <c r="G6" t="str">
-        <v>123</v>
-      </c>
-      <c r="H6" t="str">
-        <v>Diseño</v>
+        <v>ccardenas@cotelco.org</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Liderazgo y Desarrollo de equipos</v>
+        <v>1128452793</v>
       </c>
       <c r="B7" t="str">
-        <v>Camila</v>
+        <v>Est6Di</v>
       </c>
       <c r="C7" t="str">
-        <v>Est07</v>
+        <v>Diana Cecilia Castañeda Maya</v>
       </c>
       <c r="D7" t="str">
-        <v>789</v>
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E7" t="str">
-        <v>Eduardo Pacheco</v>
+        <v>DIo1</v>
       </c>
       <c r="F7" t="str">
-        <v>Doc02</v>
-      </c>
-      <c r="G7" t="str">
-        <v>123</v>
-      </c>
-      <c r="H7" t="str">
-        <v>Diseño</v>
+        <v>d.castanedamaya@gmail.com</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Sales Upgrade: Dominando Las Tecnologías</v>
+        <v>1047496837</v>
       </c>
       <c r="B8" t="str">
-        <v>Laura</v>
+        <v>Est7Di</v>
       </c>
       <c r="C8" t="str">
-        <v>Est02</v>
+        <v>Diana Marcela Campos Bueno</v>
       </c>
       <c r="D8" t="str">
-        <v>789</v>
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E8" t="str">
-        <v>Eduardo Pacheco</v>
+        <v>DIo1</v>
       </c>
       <c r="F8" t="str">
-        <v>Doc02</v>
-      </c>
-      <c r="G8" t="str">
-        <v>123</v>
-      </c>
-      <c r="H8" t="str">
-        <v>Diseño</v>
+        <v>Diadeana15@hotmail.com</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Habilidades para el siglo XXI</v>
+        <v>93414546</v>
       </c>
       <c r="B9" t="str">
-        <v>Sofia</v>
+        <v>Est8Di</v>
       </c>
       <c r="C9" t="str">
-        <v>Est08</v>
+        <v>Diego Alejandro Grajales Conde</v>
       </c>
       <c r="D9" t="str">
-        <v>789</v>
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E9" t="str">
-        <v>Ramiro Parias</v>
+        <v>DIo1</v>
       </c>
       <c r="F9" t="str">
-        <v>Doc03</v>
-      </c>
-      <c r="G9" t="str">
-        <v>123</v>
-      </c>
-      <c r="H9" t="str">
-        <v>Costos</v>
+        <v>lider.financiero@vivamosdelosbienesraices.com</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Sales Upgrade: Dominando Las Tecnologías</v>
+        <v>71352123</v>
       </c>
       <c r="B10" t="str">
-        <v>Claudia</v>
+        <v>Est9Ed</v>
       </c>
       <c r="C10" t="str">
-        <v>Est03</v>
+        <v>Edilberto Serrano Varilla</v>
       </c>
       <c r="D10" t="str">
-        <v>789</v>
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E10" t="str">
-        <v>Ramiro Parias</v>
+        <v>DIo1</v>
       </c>
       <c r="F10" t="str">
-        <v>Doc03</v>
-      </c>
-      <c r="G10" t="str">
-        <v>123</v>
-      </c>
-      <c r="H10" t="str">
-        <v>Costos</v>
+        <v>edilberto.serrano@lagoonhotel.com</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Uso estratégico de IA y transformación digital para la toma de decisiones, la eficiencia y la experiencia empresarial</v>
+        <v>73581860</v>
       </c>
       <c r="B11" t="str">
-        <v>Arturo</v>
+        <v>Est10Ed</v>
       </c>
       <c r="C11" t="str">
-        <v>Est04</v>
+        <v>Eduardo Velasquez Campo</v>
       </c>
       <c r="D11" t="str">
-        <v>789</v>
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E11" t="str">
-        <v>Ramiro Parias</v>
+        <v>DIo1</v>
       </c>
       <c r="F11" t="str">
-        <v>Doc03</v>
-      </c>
-      <c r="G11" t="str">
-        <v>123</v>
-      </c>
-      <c r="H11" t="str">
-        <v>Costos</v>
+        <v>eduardo.velasquez@lagoonhotel.com</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Control, costos y presupuestos de alimentos y bebidas</v>
+        <v>79986486</v>
       </c>
       <c r="B12" t="str">
-        <v>Arturo</v>
+        <v>Est11Ge</v>
       </c>
       <c r="C12" t="str">
-        <v>Est04</v>
+        <v>Gerardo Alberto Urrea Herrera</v>
       </c>
       <c r="D12" t="str">
-        <v>789</v>
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E12" t="str">
-        <v>Ingrid Duque</v>
+        <v>DIo1</v>
       </c>
       <c r="F12" t="str">
-        <v>Doc04</v>
-      </c>
-      <c r="G12" t="str">
-        <v>123</v>
-      </c>
-      <c r="H12" t="str">
-        <v>Analítica</v>
+        <v>REVENUE@SELVARIO36HOTEL.COM</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Creador y gestor de contenidos para empresas turisticas</v>
+        <v>1002314099</v>
       </c>
       <c r="B13" t="str">
-        <v>Laura</v>
+        <v>Est12He</v>
       </c>
       <c r="C13" t="str">
-        <v>Est02</v>
+        <v>Hernán Ricardo Carranza Montenegro</v>
       </c>
       <c r="D13" t="str">
-        <v>789</v>
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E13" t="str">
-        <v>Ingrid Duque</v>
+        <v>DIo1</v>
       </c>
       <c r="F13" t="str">
-        <v>Doc04</v>
-      </c>
-      <c r="G13" t="str">
-        <v>123</v>
-      </c>
-      <c r="H13" t="str">
-        <v>Analítica</v>
+        <v>hernancarranza560@gmail.com</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>IA y estrategia digital para el tiempo compartido</v>
+        <v>96352560</v>
       </c>
       <c r="B14" t="str">
-        <v>María</v>
+        <v>Est13Hu</v>
       </c>
       <c r="C14" t="str">
-        <v>Est09</v>
+        <v>Humberto Sánchez Cedeño</v>
       </c>
       <c r="D14" t="str">
-        <v>789</v>
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E14" t="str">
-        <v>Ingrid Duque</v>
+        <v>DIo1</v>
       </c>
       <c r="F14" t="str">
-        <v>Doc04</v>
-      </c>
-      <c r="G14" t="str">
-        <v>123</v>
-      </c>
-      <c r="H14" t="str">
-        <v>Analítica</v>
+        <v>humberto.sanchez01@est.uexternado.edu.co</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Sales Upgrade: Dominando Las Tecnologías</v>
+        <v>15512508</v>
       </c>
       <c r="B15" t="str">
-        <v>Arturo</v>
+        <v>Est14Ja</v>
       </c>
       <c r="C15" t="str">
-        <v>Est04</v>
+        <v>Jaime Toro Castillo</v>
       </c>
       <c r="D15" t="str">
-        <v>789</v>
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E15" t="str">
-        <v>Ingrid Duque</v>
+        <v>DIo1</v>
       </c>
       <c r="F15" t="str">
-        <v>Doc04</v>
-      </c>
-      <c r="G15" t="str">
-        <v>123</v>
-      </c>
-      <c r="H15" t="str">
-        <v>Analítica</v>
+        <v>gerencia@cafehotel.com.co</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Analítica de negocios de Alojamiento</v>
+        <v>73155986</v>
       </c>
       <c r="B16" t="str">
-        <v>Jonatan</v>
+        <v>Est15Jo</v>
       </c>
       <c r="C16" t="str">
-        <v>Est10</v>
+        <v>Jorge Miguel Najera Guerrero</v>
       </c>
       <c r="D16" t="str">
-        <v>789</v>
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E16" t="str">
-        <v>Camilo Ayala</v>
+        <v>DIo1</v>
       </c>
       <c r="F16" t="str">
-        <v>Doc05</v>
-      </c>
-      <c r="G16" t="str">
-        <v>123</v>
-      </c>
-      <c r="H16" t="str">
-        <v>Normatividad</v>
+        <v>Contralorgeneral@santosdepiedra.com.co</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Innovación tecnológica aplicada al sector turístico</v>
+        <v>1032438159</v>
       </c>
       <c r="B17" t="str">
-        <v>Claudia</v>
+        <v>Est16Ju</v>
       </c>
       <c r="C17" t="str">
-        <v>Est03</v>
+        <v>Juan Camilo Lovera Peña</v>
       </c>
       <c r="D17" t="str">
-        <v>789</v>
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E17" t="str">
-        <v>Camilo Ayala</v>
+        <v>DIo1</v>
       </c>
       <c r="F17" t="str">
-        <v>Doc05</v>
-      </c>
-      <c r="G17" t="str">
-        <v>123</v>
-      </c>
-      <c r="H17" t="str">
-        <v>Normatividad</v>
+        <v>gerencia@vivamosdelosbienesraices.com</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Logística, administración financiera y evaluación de eventos</v>
+        <v>1022366232</v>
       </c>
       <c r="B18" t="str">
-        <v>Heither</v>
+        <v>Est17Ju</v>
       </c>
       <c r="C18" t="str">
-        <v>Est05</v>
+        <v>Juan David Morales Corredor</v>
       </c>
       <c r="D18" t="str">
-        <v>789</v>
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E18" t="str">
-        <v>Camilo Ayala</v>
+        <v>DIo1</v>
       </c>
       <c r="F18" t="str">
-        <v>Doc05</v>
-      </c>
-      <c r="G18" t="str">
-        <v>123</v>
-      </c>
-      <c r="H18" t="str">
-        <v>Normatividad</v>
+        <v>REVENUE@V-GRANDHOTELS.COM</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Revenue management en la industria del Alojamiento</v>
+        <v>1144087674</v>
       </c>
       <c r="B19" t="str">
-        <v>David</v>
+        <v>Est18Ju</v>
       </c>
       <c r="C19" t="str">
-        <v>Est01</v>
+        <v>Juan Felipe Salgado</v>
       </c>
       <c r="D19" t="str">
-        <v>987</v>
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E19" t="str">
-        <v>Camilo Ayala</v>
+        <v>DIo1</v>
       </c>
       <c r="F19" t="str">
-        <v>Doc05</v>
-      </c>
-      <c r="G19" t="str">
-        <v>123</v>
-      </c>
-      <c r="H19" t="str">
-        <v>Normatividad</v>
+        <v>biosalgology2@gmail.com</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Sales Upgrade: Dominando Las Tecnologías</v>
+        <v>1039448085</v>
       </c>
       <c r="B20" t="str">
-        <v>Heither</v>
+        <v>Est19Ju</v>
       </c>
       <c r="C20" t="str">
-        <v>Est05</v>
+        <v>Juanita Escobar Vélez</v>
       </c>
       <c r="D20" t="str">
-        <v>789</v>
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E20" t="str">
-        <v>Camilo Ayala</v>
+        <v>DIo1</v>
       </c>
       <c r="F20" t="str">
-        <v>Doc05</v>
-      </c>
-      <c r="G20" t="str">
-        <v>123</v>
-      </c>
-      <c r="H20" t="str">
-        <v>Normatividad</v>
+        <v>juanita.escobar@eehoteles.com</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>1047444463</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Est20La</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Laura Alexandra Cuello Carbonell</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="E21" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="F21" t="str">
+        <v>cartagena.apartments1@gmail.com</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>34325204</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Est21Le</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Leydi Viviana Rivera Bastidas</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="E22" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Dadministrativo.cali@azorhoteles.com</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>1047421156</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Est22Lu</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Luis Alberto Ricaurte Barón</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="E23" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Lricaurte@doradoplaza.com</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>1083002984</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Est23Ma</v>
+      </c>
+      <c r="C24" t="str">
+        <v>María Alejandra Linero Quintana</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="E24" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Analista.datos@zuana.com.co</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>42074897</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Est24Ma</v>
+      </c>
+      <c r="C25" t="str">
+        <v>María Cecilia Jiménez</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="E25" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="F25" t="str">
+        <v>maria.jimenez@hotmail.com</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>45555715</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Est25Ma</v>
+      </c>
+      <c r="C26" t="str">
+        <v>María Ines Osorio Diaz</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="E26" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="F26" t="str">
+        <v>finanzas@wyndhamgardencartagena.com</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>1032506029</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Est26Ma</v>
+      </c>
+      <c r="C27" t="str">
+        <v>María Teresa Esteban</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="E27" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="F27" t="str">
+        <v>mariat.esteban@habitelhotels.com</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>1144194072</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Est27Na</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Natalia Echeverri Cardona</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="E28" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Gerenciamsciudadjardin@hotelesms.com</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>1006036595</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Est28Sa</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Santiago Muñoz Fajardo</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="E29" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="F29" t="str">
+        <v>samufao107@gmail.com</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>1144179760</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Est29St</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Stiven Hernández Romero</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="E30" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="F30" t="str">
+        <v>stiven.hernandez@hilton.com</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>66907448</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Est30Vi</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Viviana Castro Hoyos</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="E31" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="F31" t="str">
+        <v>viviana.castro@hotelobeliscocali.com</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F31"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Usuario</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Contraseña</v>
+      </c>
+      <c r="C1" t="str">
+        <v>NOMBRE</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Código programa</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Programa asignado</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Materia</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Horas</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Fechas de clases</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Doc01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>SA&amp;_01_TO</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Sandra Lorena Tovar</v>
+      </c>
+      <c r="D2" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Introducción a la estrategia de datos</v>
+      </c>
+      <c r="G2">
+        <v>12</v>
+      </c>
+      <c r="H2" t="str">
+        <v>07, 08, 09, 14, 15, 16 de abril 2026</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Doc02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>EM&amp;_02_CA</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Emma Camargo</v>
+      </c>
+      <c r="D3" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Protección de datos</v>
+      </c>
+      <c r="G3">
+        <v>8</v>
+      </c>
+      <c r="H3" t="str">
+        <v>21, 22, 23, 28 de abril 2026</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Doc03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>WI&amp;_03_ES</v>
+      </c>
+      <c r="C4" t="str">
+        <v>William Rodrigo Escobar</v>
+      </c>
+      <c r="D4" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Inteligencia de Negocios para establecimientos de alojamiento</v>
+      </c>
+      <c r="G4">
+        <v>18</v>
+      </c>
+      <c r="H4" t="str">
+        <v>29, 30 de abril 2026, 05, 06, 07, 12, 13, 14, 19, 20 de mayo 2026</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Doc04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>NA&amp;_04_AM</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Natalia Contreras Amaya</v>
+      </c>
+      <c r="D5" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Inteligencia de Negocios para establecimientos de alojamiento</v>
+      </c>
+      <c r="G5">
+        <v>20</v>
+      </c>
+      <c r="H5" t="str">
+        <v>21, 26, 27, 28 de mayo 2026 y 02, 03, 04, 09, 10, 11 de junio 2026</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Doc05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>JO&amp;_05_PE</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Jonathan Andrés Pérez López</v>
+      </c>
+      <c r="D6" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Analítica de Negocios: Power Query y estadística descriptiva aplicada</v>
+      </c>
+      <c r="G6">
+        <v>10</v>
+      </c>
+      <c r="H6" t="str">
+        <v>16, 17, 18, 23, 24 de junio 2026</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Doc05</v>
+      </c>
+      <c r="B7" t="str">
+        <v>JO&amp;_05_PE</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Jonathan Andrés Pérez López</v>
+      </c>
+      <c r="D7" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Analítica de Negocios: Estadística Inferencial para decisiones comerciales</v>
+      </c>
+      <c r="G7">
+        <v>6</v>
+      </c>
+      <c r="H7" t="str">
+        <v>25, 30 de junio 2026 y 01 de julio 2026</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Doc07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>ED&amp;_07_SU</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Eduárez</v>
+      </c>
+      <c r="D8" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Analítica de Negocios: Tecnología de datos en turismo</v>
+      </c>
+      <c r="G8">
+        <v>14</v>
+      </c>
+      <c r="H8" t="str">
+        <v>02, 07, 08, 09, 14, 15, 16 de julio 2026</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Doc08</v>
+      </c>
+      <c r="B9" t="str">
+        <v>SA&amp;_08_TO</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Sandra Lorena Tovar</v>
+      </c>
+      <c r="D9" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Analítica de Negocios: BI sin código: Introducción a Power BI / Looker</v>
+      </c>
+      <c r="G9">
+        <v>14</v>
+      </c>
+      <c r="H9" t="str">
+        <v>21, 22, 23, 28, 29, 30 de julio 2026 y 04 de agosto 2026</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Doc09</v>
+      </c>
+      <c r="B10" t="str">
+        <v>MA&amp;_09_SA</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Mario Sánchez</v>
+      </c>
+      <c r="D10" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Analítica de Negocios: IA como copiloto de la analítica turística</v>
+      </c>
+      <c r="G10">
+        <v>16</v>
+      </c>
+      <c r="H10" t="str">
+        <v>05, 06, 11, 12, 13, 18, 19, 20 de agosto 2026</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Usuario</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Contraseña</v>
+      </c>
+      <c r="C1" t="str">
+        <v>NOMBRE</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Admin01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>AC_&amp;jo*2026</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Academica Turismo</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: add new students to excel
</commit_message>
<xml_diff>
--- a/data/journey.xlsx
+++ b/data/journey.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F33"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1021,9 +1021,43 @@
         <v>viviana.castro@hotelobeliscocali.com</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32">
+        <v>1130683651</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Est31Da</v>
+      </c>
+      <c r="C32" t="str">
+        <v>ACOSTA GAVIRIA DARLY JOHANNA</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="E32" t="str">
+        <v>DIo1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <v>1107077642</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Est32Fo</v>
+      </c>
+      <c r="C33" t="str">
+        <v>RAMIREZ FORY NATALI</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="E33" t="str">
+        <v>DIo1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F33"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add new students Est33-Est34 and update teacher hours to 120h
</commit_message>
<xml_diff>
--- a/data/journey.xlsx
+++ b/data/journey.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F35"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1022,14 +1022,14 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32">
+      <c r="A32" t="str">
         <v>1130683651</v>
       </c>
       <c r="B32" t="str">
         <v>Est31Da</v>
       </c>
       <c r="C32" t="str">
-        <v>ACOSTA GAVIRIA DARLY JOHANNA</v>
+        <v>DARLY JOHANNA ACOSTA GAVIRIA</v>
       </c>
       <c r="D32" t="str">
         <v>Diplomado en Analítica de Negocios de Alojamiento</v>
@@ -1037,27 +1037,73 @@
       <c r="E32" t="str">
         <v>DIo1</v>
       </c>
+      <c r="F32" t="str">
+        <v>darly.acosta@gmail.com</v>
+      </c>
     </row>
     <row r="33">
-      <c r="A33">
+      <c r="A33" t="str">
         <v>1107077642</v>
       </c>
       <c r="B33" t="str">
         <v>Est32Fo</v>
       </c>
       <c r="C33" t="str">
-        <v>RAMIREZ FORY NATALI</v>
+        <v>NATALI RAMIREZ FORY</v>
       </c>
       <c r="D33" t="str">
         <v>Diplomado en Analítica de Negocios de Alojamiento</v>
       </c>
       <c r="E33" t="str">
         <v>DIo1</v>
+      </c>
+      <c r="F33" t="str">
+        <v>natali.ramirez@gmail.com</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>52423831</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Est33Cl</v>
+      </c>
+      <c r="C34" t="str">
+        <v>CLAUDIA XIMENA CEPEDA HIDALGO</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="E34" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="F34" t="str">
+        <v>claudia.cepeda@gmail.com</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>79954231</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Est34He</v>
+      </c>
+      <c r="C35" t="str">
+        <v>HEITHER ALEXANDER OMAÑA</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Diplomado en Analítica de Negocios de Alojamiento</v>
+      </c>
+      <c r="E35" t="str">
+        <v>DIo1</v>
+      </c>
+      <c r="F35" t="str">
+        <v>heither.omana@gmail.com</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F35"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1164,7 +1210,7 @@
         <v>Inteligencia de Negocios para establecimientos de alojamiento</v>
       </c>
       <c r="G4">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H4" t="str">
         <v>29, 30 de abril 2026, 05, 06, 07, 12, 13, 14, 19, 20 de mayo 2026</v>
@@ -1256,7 +1302,7 @@
         <v>ED&amp;_07_SU</v>
       </c>
       <c r="C8" t="str">
-        <v>Eduárez</v>
+        <v>Eduardo Suárez</v>
       </c>
       <c r="D8" t="str">
         <v>DIo1</v>

</xml_diff>